<commit_message>
replacement data for healthcare
</commit_message>
<xml_diff>
--- a/cert-data/Healthcare-Certification-Report-09.22.2026.xlsx
+++ b/cert-data/Healthcare-Certification-Report-09.22.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://konicaminoltanam-my.sharepoint.com/personal/rnesimi_kmbsus_com/Documents/Dashboard Reports/Healthcare Dashboard Reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{514B226B-F3E3-46A6-853F-6F49CE7CAE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3EAC62F-0280-470C-B735-1F72D6FBFFF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9760" yWindow="10690" windowWidth="19420" windowHeight="11500" xr2:uid="{DC5E560D-579C-485D-825F-94F306B9108B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1157" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1163" uniqueCount="303">
   <si>
     <t>User</t>
   </si>
@@ -432,12 +432,6 @@
   </si>
   <si>
     <t>rfielding@kmbs.konicaminolta.us</t>
-  </si>
-  <si>
-    <t>East</t>
-  </si>
-  <si>
-    <t>Florida</t>
   </si>
   <si>
     <t>Oldsmar</t>
@@ -1909,7 +1903,6 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3DB49C0E-B689-40D7-AF80-6540B72913D2}" name="Table1" displayName="Table1" ref="A1:U71" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:U71" xr:uid="{3DB49C0E-B689-40D7-AF80-6540B72913D2}"/>
   <tableColumns count="21">
     <tableColumn id="1" xr3:uid="{7E27C642-CD96-4E29-8515-090A1E2597B4}" name="User" dataDxfId="20"/>
     <tableColumn id="21" xr3:uid="{50452B11-87F7-47DB-9B0B-60BC2C16FB02}" name="Active Users" dataDxfId="19"/>
@@ -3555,6 +3548,12 @@
       <c r="F20" s="2" t="s">
         <v>121</v>
       </c>
+      <c r="G20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="J20" s="2" t="s">
         <v>28</v>
       </c>
@@ -3612,6 +3611,12 @@
       <c r="F21" s="2" t="s">
         <v>121</v>
       </c>
+      <c r="G21" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="J21" s="2" t="s">
         <v>28</v>
       </c>
@@ -3670,13 +3675,13 @@
         <v>121</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>28</v>
@@ -3727,13 +3732,19 @@
         <v>36</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>121</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>28</v>
@@ -3781,16 +3792,16 @@
         <v>21</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>140</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>26</v>
@@ -3847,16 +3858,16 @@
         <v>21</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>26</v>
@@ -3913,16 +3924,16 @@
         <v>21</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E26" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>26</v>
@@ -3979,16 +3990,16 @@
         <v>21</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>26</v>
@@ -4048,13 +4059,13 @@
         <v>70</v>
       </c>
       <c r="D28" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>26</v>
@@ -4111,16 +4122,16 @@
         <v>21</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>26</v>
@@ -4177,16 +4188,16 @@
         <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>50</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>26</v>
@@ -4243,16 +4254,16 @@
         <v>21</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="F31" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>26</v>
@@ -4267,13 +4278,13 @@
         <v>126</v>
       </c>
       <c r="K31" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="M31" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="N31" s="2" t="s">
         <v>32</v>
@@ -4309,16 +4320,16 @@
         <v>21</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>171</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>26</v>
@@ -4375,16 +4386,16 @@
         <v>21</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>175</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>26</v>
@@ -4441,16 +4452,16 @@
         <v>21</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>177</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>26</v>
@@ -4507,16 +4518,16 @@
         <v>21</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>182</v>
-      </c>
       <c r="F35" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>26</v>
@@ -4573,16 +4584,16 @@
         <v>21</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D36" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="F36" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>26</v>
@@ -4597,13 +4608,13 @@
         <v>126</v>
       </c>
       <c r="K36" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="M36" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="N36" s="2" t="s">
         <v>32</v>
@@ -4639,16 +4650,16 @@
         <v>21</v>
       </c>
       <c r="C37" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>188</v>
-      </c>
       <c r="F37" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>26</v>
@@ -4705,16 +4716,16 @@
         <v>21</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>191</v>
-      </c>
       <c r="F38" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>26</v>
@@ -4771,16 +4782,16 @@
         <v>21</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E39" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>194</v>
-      </c>
       <c r="F39" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>26</v>
@@ -4837,16 +4848,16 @@
         <v>21</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>197</v>
-      </c>
       <c r="F40" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>26</v>
@@ -4903,16 +4914,16 @@
         <v>21</v>
       </c>
       <c r="C41" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="F41" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>26</v>
@@ -4969,16 +4980,16 @@
         <v>21</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>204</v>
-      </c>
       <c r="F42" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>26</v>
@@ -5035,16 +5046,16 @@
         <v>21</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>207</v>
-      </c>
       <c r="F43" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>26</v>
@@ -5101,16 +5112,16 @@
         <v>21</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>210</v>
-      </c>
       <c r="F44" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>26</v>
@@ -5167,16 +5178,16 @@
         <v>21</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="F45" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>214</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>26</v>
@@ -5233,16 +5244,16 @@
         <v>21</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="D46" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>217</v>
-      </c>
       <c r="F46" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>26</v>
@@ -5299,16 +5310,16 @@
         <v>21</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>26</v>
@@ -5365,16 +5376,16 @@
         <v>21</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="E48" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>222</v>
-      </c>
       <c r="F48" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>26</v>
@@ -5431,16 +5442,16 @@
         <v>21</v>
       </c>
       <c r="C49" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D49" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>225</v>
-      </c>
       <c r="F49" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>26</v>
@@ -5497,16 +5508,16 @@
         <v>21</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="D50" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>228</v>
-      </c>
       <c r="F50" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G50" s="2" t="s">
         <v>26</v>
@@ -5563,16 +5574,16 @@
         <v>21</v>
       </c>
       <c r="C51" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E51" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D51" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>231</v>
-      </c>
       <c r="F51" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G51" s="2" t="s">
         <v>26</v>
@@ -5629,16 +5640,16 @@
         <v>21</v>
       </c>
       <c r="C52" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="E52" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="D52" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="F52" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G52" s="2" t="s">
         <v>26</v>
@@ -5653,13 +5664,13 @@
         <v>126</v>
       </c>
       <c r="K52" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="L52" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="M52" s="2" t="s">
         <v>165</v>
-      </c>
-      <c r="L52" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="M52" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="N52" s="2" t="s">
         <v>32</v>
@@ -5695,16 +5706,16 @@
         <v>21</v>
       </c>
       <c r="C53" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E53" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>237</v>
-      </c>
       <c r="F53" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G53" s="2" t="s">
         <v>26</v>
@@ -5761,16 +5772,16 @@
         <v>21</v>
       </c>
       <c r="C54" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="D54" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>240</v>
-      </c>
       <c r="F54" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="G54" s="2" t="s">
         <v>26</v>
@@ -5827,16 +5838,16 @@
         <v>21</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G55" s="2" t="s">
         <v>26</v>
@@ -5893,16 +5904,16 @@
         <v>21</v>
       </c>
       <c r="C56" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E56" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="D56" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>245</v>
-      </c>
       <c r="F56" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="G56" s="2" t="s">
         <v>26</v>
@@ -5959,16 +5970,16 @@
         <v>21</v>
       </c>
       <c r="C57" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="E57" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="D57" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>248</v>
-      </c>
       <c r="F57" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G57" s="2" t="s">
         <v>26</v>
@@ -6025,16 +6036,16 @@
         <v>21</v>
       </c>
       <c r="C58" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="E58" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="D58" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>251</v>
-      </c>
       <c r="F58" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>26</v>
@@ -6091,16 +6102,16 @@
         <v>21</v>
       </c>
       <c r="C59" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E59" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="D59" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>254</v>
-      </c>
       <c r="F59" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>26</v>
@@ -6112,13 +6123,13 @@
         <v>39</v>
       </c>
       <c r="J59" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="L59" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="K59" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="L59" s="2" t="s">
-        <v>257</v>
       </c>
       <c r="M59" s="2" t="s">
         <v>25</v>
@@ -6157,16 +6168,16 @@
         <v>21</v>
       </c>
       <c r="C60" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E60" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>260</v>
-      </c>
       <c r="F60" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>26</v>
@@ -6223,37 +6234,37 @@
         <v>21</v>
       </c>
       <c r="C61" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E61" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="F61" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="G61" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="F61" s="2" t="s">
+      <c r="H61" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="G61" s="2" t="s">
+      <c r="I61" s="2" t="s">
         <v>265</v>
-      </c>
-      <c r="H61" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="I61" s="2" t="s">
-        <v>267</v>
       </c>
       <c r="J61" s="2" t="s">
         <v>70</v>
       </c>
       <c r="K61" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="L61" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="M61" s="2" t="s">
         <v>268</v>
-      </c>
-      <c r="L61" s="2" t="s">
-        <v>269</v>
-      </c>
-      <c r="M61" s="2" t="s">
-        <v>270</v>
       </c>
       <c r="N61" s="2" t="s">
         <v>32</v>
@@ -6269,7 +6280,7 @@
       </c>
       <c r="R61" s="1"/>
       <c r="T61" s="11" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="62" spans="1:21">
@@ -6280,16 +6291,16 @@
         <v>21</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>26</v>
@@ -6326,7 +6337,7 @@
       </c>
       <c r="R62" s="1"/>
       <c r="T62" s="11" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="63" spans="1:21">
@@ -6337,13 +6348,13 @@
         <v>21</v>
       </c>
       <c r="C63" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>274</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>276</v>
       </c>
       <c r="F63" s="2" t="s">
         <v>25</v>
@@ -6383,7 +6394,7 @@
       </c>
       <c r="R63" s="9"/>
       <c r="T63" s="11" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="64" spans="1:21">
@@ -6394,16 +6405,16 @@
         <v>21</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E64" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="D64" s="2" t="s">
-        <v>278</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>279</v>
-      </c>
       <c r="F64" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>26</v>
@@ -6415,13 +6426,13 @@
         <v>39</v>
       </c>
       <c r="J64" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="L64" s="2" t="s">
         <v>280</v>
-      </c>
-      <c r="K64" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="L64" s="2" t="s">
-        <v>282</v>
       </c>
       <c r="M64" s="2" t="s">
         <v>25</v>
@@ -6460,16 +6471,16 @@
         <v>21</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>26</v>
@@ -6507,14 +6518,14 @@
       <c r="R65" s="1"/>
       <c r="S65" s="4"/>
       <c r="T65" s="11" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="U65" s="4"/>
       <c r="X65" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="AD65" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="66" spans="1:30">
@@ -6525,16 +6536,16 @@
         <v>21</v>
       </c>
       <c r="C66" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="E66" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="D66" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>289</v>
-      </c>
       <c r="F66" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>26</v>
@@ -6588,16 +6599,16 @@
         <v>21</v>
       </c>
       <c r="C67" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="D67" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>292</v>
-      </c>
       <c r="F67" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>26</v>
@@ -6651,16 +6662,16 @@
         <v>21</v>
       </c>
       <c r="C68" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E68" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>295</v>
-      </c>
       <c r="F68" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G68" s="2" t="s">
         <v>26</v>
@@ -6714,16 +6725,16 @@
         <v>21</v>
       </c>
       <c r="C69" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D69" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>298</v>
-      </c>
       <c r="F69" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>26</v>
@@ -6777,16 +6788,16 @@
         <v>21</v>
       </c>
       <c r="C70" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E70" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>301</v>
-      </c>
       <c r="F70" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G70" s="2" t="s">
         <v>26</v>
@@ -6843,13 +6854,13 @@
         <v>61</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>26</v>
@@ -6897,7 +6908,7 @@
     </row>
     <row r="73" spans="1:30">
       <c r="S73" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>